<commit_message>
Atualiza planilha diária de leads e conformidade
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1167"/>
+  <dimension ref="A1:L1197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56343,10 +56343,8 @@
         </is>
       </c>
       <c r="H1147" t="inlineStr"/>
-      <c r="I1147" t="inlineStr">
-        <is>
-          <t>556193656589</t>
-        </is>
+      <c r="I1147" t="n">
+        <v>556193656589</v>
       </c>
       <c r="J1147" t="inlineStr"/>
       <c r="K1147" t="n">
@@ -56395,10 +56393,8 @@
         </is>
       </c>
       <c r="H1148" t="inlineStr"/>
-      <c r="I1148" t="inlineStr">
-        <is>
-          <t>5561993041166</t>
-        </is>
+      <c r="I1148" t="n">
+        <v>5561993041166</v>
       </c>
       <c r="J1148" t="inlineStr"/>
       <c r="K1148" t="n">
@@ -56543,10 +56539,8 @@
         </is>
       </c>
       <c r="H1151" t="inlineStr"/>
-      <c r="I1151" t="inlineStr">
-        <is>
-          <t>5561984048581</t>
-        </is>
+      <c r="I1151" t="n">
+        <v>5561984048581</v>
       </c>
       <c r="J1151" t="inlineStr"/>
       <c r="K1151" t="n">
@@ -56595,10 +56589,8 @@
         </is>
       </c>
       <c r="H1152" t="inlineStr"/>
-      <c r="I1152" t="inlineStr">
-        <is>
-          <t>5511976396153</t>
-        </is>
+      <c r="I1152" t="n">
+        <v>5511976396153</v>
       </c>
       <c r="J1152" t="inlineStr"/>
       <c r="K1152" t="n">
@@ -56695,10 +56687,8 @@
         </is>
       </c>
       <c r="H1154" t="inlineStr"/>
-      <c r="I1154" t="inlineStr">
-        <is>
-          <t>5521999850091</t>
-        </is>
+      <c r="I1154" t="n">
+        <v>5521999850091</v>
       </c>
       <c r="J1154" t="inlineStr"/>
       <c r="K1154" t="n">
@@ -56747,10 +56737,8 @@
         </is>
       </c>
       <c r="H1155" t="inlineStr"/>
-      <c r="I1155" t="inlineStr">
-        <is>
-          <t>5561992926161</t>
-        </is>
+      <c r="I1155" t="n">
+        <v>5561992926161</v>
       </c>
       <c r="J1155" t="inlineStr"/>
       <c r="K1155" t="n">
@@ -56799,10 +56787,8 @@
         </is>
       </c>
       <c r="H1156" t="inlineStr"/>
-      <c r="I1156" t="inlineStr">
-        <is>
-          <t>556196811386</t>
-        </is>
+      <c r="I1156" t="n">
+        <v>556196811386</v>
       </c>
       <c r="J1156" t="inlineStr"/>
       <c r="K1156" t="n">
@@ -56851,10 +56837,8 @@
         </is>
       </c>
       <c r="H1157" t="inlineStr"/>
-      <c r="I1157" t="inlineStr">
-        <is>
-          <t>5561992541042</t>
-        </is>
+      <c r="I1157" t="n">
+        <v>5561992541042</v>
       </c>
       <c r="J1157" t="inlineStr"/>
       <c r="K1157" t="n">
@@ -56999,10 +56983,8 @@
         </is>
       </c>
       <c r="H1160" t="inlineStr"/>
-      <c r="I1160" t="inlineStr">
-        <is>
-          <t>5562981942470</t>
-        </is>
+      <c r="I1160" t="n">
+        <v>5562981942470</v>
       </c>
       <c r="J1160" t="inlineStr"/>
       <c r="K1160" t="n">
@@ -57147,10 +57129,8 @@
         </is>
       </c>
       <c r="H1163" t="inlineStr"/>
-      <c r="I1163" t="inlineStr">
-        <is>
-          <t>5562982254507</t>
-        </is>
+      <c r="I1163" t="n">
+        <v>5562982254507</v>
       </c>
       <c r="J1163" t="inlineStr"/>
       <c r="K1163" t="n">
@@ -57354,6 +57334,1478 @@
         </is>
       </c>
     </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>Clínica Amme</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>https://grupoammare.com.br</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr"/>
+      <c r="I1168" t="inlineStr"/>
+      <c r="J1168" t="inlineStr"/>
+      <c r="K1168" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1168" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>Pronto Atendimento</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>https://www.hospitalvitoriaapart.com.br</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr"/>
+      <c r="I1169" t="inlineStr"/>
+      <c r="J1169" t="inlineStr"/>
+      <c r="K1169" t="n">
+        <v>88</v>
+      </c>
+      <c r="L1169" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>Clínica Kairós</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>https://clinicakairosvitoria.com.br</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr"/>
+      <c r="I1170" t="inlineStr"/>
+      <c r="J1170" t="inlineStr"/>
+      <c r="K1170" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1170" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Conheça Vitória / ES</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>https://attitudepromo.iweventos.com.br</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr"/>
+      <c r="I1171" t="inlineStr"/>
+      <c r="J1171" t="inlineStr"/>
+      <c r="K1171" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1171" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>FORMAN Medicina</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>https://formanmedicina.com.br</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr"/>
+      <c r="I1172" t="inlineStr"/>
+      <c r="J1172" t="inlineStr"/>
+      <c r="K1172" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1172" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>Psicóloga em Vitória, ES</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>https://psicologagiulianadepaula.com.br</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr"/>
+      <c r="I1173" t="inlineStr"/>
+      <c r="J1173" t="inlineStr"/>
+      <c r="K1173" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1173" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>Os currículos da Educação Física na educação infantil em ...</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>https://periodicos.pucpr.br</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr"/>
+      <c r="I1174" t="inlineStr"/>
+      <c r="J1174" t="inlineStr"/>
+      <c r="K1174" t="n">
+        <v>53</v>
+      </c>
+      <c r="L1174" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>EXPERIÊNCIAS NA EDUCAÇÃO INFANTIL DE VITÓRIA/ES</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>https://portalespiral.cp2.g12.br</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr"/>
+      <c r="I1175" t="inlineStr"/>
+      <c r="J1175" t="inlineStr"/>
+      <c r="K1175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1175" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>[PDF] atuação do fisioterapeuta na atenção na básica, na perspectiva ...</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>https://revista.faesa.br</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr"/>
+      <c r="I1176" t="inlineStr"/>
+      <c r="J1176" t="inlineStr"/>
+      <c r="K1176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1176" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>Clinica Sagrada Família</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>https://clinicamedsagradafamilia.com.br</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr"/>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>5531975954885</t>
+        </is>
+      </c>
+      <c r="J1177" t="inlineStr"/>
+      <c r="K1177" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1177" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>https://www.clinicaaima.com.br</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr"/>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>5531999997188</t>
+        </is>
+      </c>
+      <c r="J1178" t="inlineStr"/>
+      <c r="K1178" t="n">
+        <v>76</v>
+      </c>
+      <c r="L1178" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>Clinica Médica São Paulo - Belo Horizonte - MG</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>https://www.climesp.com.br</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr"/>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>5531999345416</t>
+        </is>
+      </c>
+      <c r="J1179" t="inlineStr"/>
+      <c r="K1179" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1179" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>Aspemed</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>https://aspemed.com.br</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr"/>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>5531973133014</t>
+        </is>
+      </c>
+      <c r="J1180" t="inlineStr"/>
+      <c r="K1180" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1180" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>Contato</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>https://www.clinicamarcosandrade.com</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr"/>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>5531971622529</t>
+        </is>
+      </c>
+      <c r="J1181" t="inlineStr"/>
+      <c r="K1181" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1181" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>Clínica de Psicologia PUC Minas</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>https://www.pucminas.br</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr"/>
+      <c r="I1182" t="inlineStr"/>
+      <c r="J1182" t="inlineStr"/>
+      <c r="K1182" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1182" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>32 treinadores e professores de esporte em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>https://www.suasaulasparticulares.com.br</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr"/>
+      <c r="I1183" t="inlineStr"/>
+      <c r="J1183" t="inlineStr"/>
+      <c r="K1183" t="n">
+        <v>90</v>
+      </c>
+      <c r="L1183" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>Personal Trainers em Belo Horizonte, MG</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>https://www.supertrainers.com.br</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr"/>
+      <c r="I1184" t="inlineStr"/>
+      <c r="J1184" t="inlineStr"/>
+      <c r="K1184" t="n">
+        <v>70</v>
+      </c>
+      <c r="L1184" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>Top 10 Academias de BH: Onde Treinar na Capital MineiraAcademias em Belo Horizonte, MG, Brasil</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>https://overallgymbh.com.br</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr"/>
+      <c r="I1185" t="inlineStr"/>
+      <c r="J1185" t="inlineStr"/>
+      <c r="K1185" t="n">
+        <v>60</v>
+      </c>
+      <c r="L1185" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>Dental Borges</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>https://dentalborges.com.br</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr"/>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>552138721919</t>
+        </is>
+      </c>
+      <c r="J1186" t="inlineStr"/>
+      <c r="K1186" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1186" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>Revista Científica do CRO-RJ (Rio de Janeiro Dental Journal)</t>
+        </is>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>https://revcientifica.cro-rj.org.br</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr"/>
+      <c r="I1187" t="inlineStr"/>
+      <c r="J1187" t="inlineStr"/>
+      <c r="K1187" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1187" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>Dentista em Rio de Janeiro com Convênio</t>
+        </is>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>https://www.encontreseudentista.com.br</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr"/>
+      <c r="I1188" t="inlineStr"/>
+      <c r="J1188" t="inlineStr"/>
+      <c r="K1188" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1188" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>Sorriso Carioca</t>
+        </is>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>https://www.victorhugoalmeida.com.br</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr"/>
+      <c r="I1189" t="inlineStr"/>
+      <c r="J1189" t="inlineStr"/>
+      <c r="K1189" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1189" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>Odonto Premier: Home</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>https://clinicaodontopremier.com.br</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr"/>
+      <c r="I1190" t="inlineStr"/>
+      <c r="J1190" t="inlineStr"/>
+      <c r="K1190" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1190" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>Nova Odonto</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>https://novaodontorj.com</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr"/>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>5521984158201</t>
+        </is>
+      </c>
+      <c r="J1191" t="inlineStr"/>
+      <c r="K1191" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1191" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>Psicólogos Sem Fronteiras</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>https://psf.org.br</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr"/>
+      <c r="I1192" t="inlineStr"/>
+      <c r="J1192" t="inlineStr"/>
+      <c r="K1192" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1192" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>SPA Serviços</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>https://www.psi.puc-rio.br</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr"/>
+      <c r="I1193" t="inlineStr"/>
+      <c r="J1193" t="inlineStr"/>
+      <c r="K1193" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1193" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>Psicologia para Adultos</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>https://terapiascopacabana.com.br</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr"/>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>5521995673175</t>
+        </is>
+      </c>
+      <c r="J1194" t="inlineStr"/>
+      <c r="K1194" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1194" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>Cadastro Nacional de Profissionais de Psicologia</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>https://cadastro.cfp.org.br</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr"/>
+      <c r="I1195" t="inlineStr"/>
+      <c r="J1195" t="inlineStr"/>
+      <c r="K1195" t="n">
+        <v>60</v>
+      </c>
+      <c r="L1195" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>Estudos e Pesquisas em Psicologia</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>https://www.e-publicacoes.uerj.br</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr"/>
+      <c r="I1196" t="inlineStr"/>
+      <c r="J1196" t="inlineStr"/>
+      <c r="K1196" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1196" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>Encontre seu Terapeuta</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>https://terapeutasdobrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr"/>
+      <c r="I1197" t="inlineStr"/>
+      <c r="J1197" t="inlineStr"/>
+      <c r="K1197" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1197" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Centro-Oeste, 2026-09-15)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1288"/>
+  <dimension ref="A1:L1300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62737,10 +62737,8 @@
         </is>
       </c>
       <c r="H1278" t="inlineStr"/>
-      <c r="I1278" t="inlineStr">
-        <is>
-          <t>5582000000000</t>
-        </is>
+      <c r="I1278" t="n">
+        <v>5582000000000</v>
       </c>
       <c r="J1278" t="inlineStr"/>
       <c r="K1278" t="n">
@@ -62933,10 +62931,8 @@
         </is>
       </c>
       <c r="H1282" t="inlineStr"/>
-      <c r="I1282" t="inlineStr">
-        <is>
-          <t>5508009719777</t>
-        </is>
+      <c r="I1282" t="n">
+        <v>5508009719777</v>
       </c>
       <c r="J1282" t="inlineStr"/>
       <c r="K1282" t="n">
@@ -63081,10 +63077,8 @@
         </is>
       </c>
       <c r="H1285" t="inlineStr"/>
-      <c r="I1285" t="inlineStr">
-        <is>
-          <t>5571982154282</t>
-        </is>
+      <c r="I1285" t="n">
+        <v>5571982154282</v>
       </c>
       <c r="J1285" t="inlineStr"/>
       <c r="K1285" t="n">
@@ -63133,10 +63127,8 @@
         </is>
       </c>
       <c r="H1286" t="inlineStr"/>
-      <c r="I1286" t="inlineStr">
-        <is>
-          <t>5571981354300</t>
-        </is>
+      <c r="I1286" t="n">
+        <v>5571981354300</v>
       </c>
       <c r="J1286" t="inlineStr"/>
       <c r="K1286" t="n">
@@ -63244,6 +63236,614 @@
         </is>
       </c>
     </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Brasília — Asa Sul</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>https://cefisbsb.com.br</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr"/>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>5561995092995</t>
+        </is>
+      </c>
+      <c r="J1289" t="inlineStr"/>
+      <c r="K1289" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1289" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>Centro Médico de Brasília</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>https://centromedicodebrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr"/>
+      <c r="I1290" t="inlineStr"/>
+      <c r="J1290" t="inlineStr"/>
+      <c r="K1290" t="n">
+        <v>56</v>
+      </c>
+      <c r="L1290" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>Terapia TRG em Brasília</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>https://www.espacoemocional.com.br</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr"/>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>5561995704309</t>
+        </is>
+      </c>
+      <c r="J1291" t="inlineStr"/>
+      <c r="K1291" t="n">
+        <v>59</v>
+      </c>
+      <c r="L1291" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>Escritório de Advocacia em Brasília</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>https://campospinho.adv.br</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr"/>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>5561981490953</t>
+        </is>
+      </c>
+      <c r="J1292" t="inlineStr"/>
+      <c r="K1292" t="n">
+        <v>64</v>
+      </c>
+      <c r="L1292" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>Via Médica</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>http://www.viamedica-go.com.br</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr"/>
+      <c r="I1293" t="inlineStr"/>
+      <c r="J1293" t="inlineStr"/>
+      <c r="K1293" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1293" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>Clínica Médica Particular Acessível em Goiânia e Valparaíso</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>https://www.souclinicavitta.com.br</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr"/>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>556239960505</t>
+        </is>
+      </c>
+      <c r="J1294" t="inlineStr"/>
+      <c r="K1294" t="n">
+        <v>53</v>
+      </c>
+      <c r="L1294" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>Daniel Vieira</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>https://www.danielvieirapsicologo.com.br</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr"/>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>5562999574089</t>
+        </is>
+      </c>
+      <c r="J1295" t="inlineStr"/>
+      <c r="K1295" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1295" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>Cairo Filho — Psicólogo Clínico</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>https://www.cairofilhopsi.com.br</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr"/>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>5562991674706</t>
+        </is>
+      </c>
+      <c r="J1296" t="inlineStr"/>
+      <c r="K1296" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1296" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>Terapeuta Em Goiânia</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>https://claudiabarrosterapeuta.com</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr"/>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>556282361670</t>
+        </is>
+      </c>
+      <c r="J1297" t="inlineStr"/>
+      <c r="K1297" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1297" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>Marília Martins Advocacia</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>https://mariliamartins.com.br</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr"/>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>5562994105041</t>
+        </is>
+      </c>
+      <c r="J1298" t="inlineStr"/>
+      <c r="K1298" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1298" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>Bernardes &amp; Viana Advogados</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>https://www.bevadv.com.br</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr"/>
+      <c r="I1299" t="inlineStr"/>
+      <c r="J1299" t="inlineStr"/>
+      <c r="K1299" t="n">
+        <v>64</v>
+      </c>
+      <c r="L1299" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>FEFD</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>https://fefd.ufg.br</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr"/>
+      <c r="I1300" t="inlineStr"/>
+      <c r="J1300" t="inlineStr"/>
+      <c r="K1300" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Norte, 2026-09-18)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1321"/>
+  <dimension ref="A1:L1328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64599,10 +64599,8 @@
         </is>
       </c>
       <c r="H1316" t="inlineStr"/>
-      <c r="I1316" t="inlineStr">
-        <is>
-          <t>5541988377317</t>
-        </is>
+      <c r="I1316" t="n">
+        <v>5541988377317</v>
       </c>
       <c r="J1316" t="inlineStr"/>
       <c r="K1316" t="n">
@@ -64651,10 +64649,8 @@
         </is>
       </c>
       <c r="H1317" t="inlineStr"/>
-      <c r="I1317" t="inlineStr">
-        <is>
-          <t>5541995158069</t>
-        </is>
+      <c r="I1317" t="n">
+        <v>5541995158069</v>
       </c>
       <c r="J1317" t="inlineStr"/>
       <c r="K1317" t="n">
@@ -64751,10 +64747,8 @@
         </is>
       </c>
       <c r="H1319" t="inlineStr"/>
-      <c r="I1319" t="inlineStr">
-        <is>
-          <t>5551983441433</t>
-        </is>
+      <c r="I1319" t="n">
+        <v>5551983441433</v>
       </c>
       <c r="J1319" t="inlineStr"/>
       <c r="K1319" t="n">
@@ -64803,10 +64797,8 @@
         </is>
       </c>
       <c r="H1320" t="inlineStr"/>
-      <c r="I1320" t="inlineStr">
-        <is>
-          <t>5551992639978</t>
-        </is>
+      <c r="I1320" t="n">
+        <v>5551992639978</v>
       </c>
       <c r="J1320" t="inlineStr"/>
       <c r="K1320" t="n">
@@ -64866,6 +64858,354 @@
         </is>
       </c>
     </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>DENTISTA DA FAMILIA</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>https://querobrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr"/>
+      <c r="I1322" t="inlineStr"/>
+      <c r="J1322" t="inlineStr"/>
+      <c r="K1322" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1322" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>Tobias Meireles Advogados</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>https://tobiasmeirelesadvogados.com</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr"/>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>5568992383844</t>
+        </is>
+      </c>
+      <c r="J1323" t="inlineStr"/>
+      <c r="K1323" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1323" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>Clínica Saúde Integrada</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>https://www.clinicasudeintegrada.com.br</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr"/>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>5596981388092</t>
+        </is>
+      </c>
+      <c r="J1324" t="inlineStr"/>
+      <c r="K1324" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1324" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>Clínica Odontológica em Manaus</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>https://www.sanmede.com.br</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr"/>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>559231992420</t>
+        </is>
+      </c>
+      <c r="J1325" t="inlineStr"/>
+      <c r="K1325" t="n">
+        <v>67</v>
+      </c>
+      <c r="L1325" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>VIANA &amp; BARBOSA ADVOGADOS - Advogado Trabalhista Manaus</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>https://vianaebarbosaadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr"/>
+      <c r="I1326" t="inlineStr"/>
+      <c r="J1326" t="inlineStr"/>
+      <c r="K1326" t="n">
+        <v>55</v>
+      </c>
+      <c r="L1326" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>Vestibular em Educação Física</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://www.unilasalle.edu.br</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr"/>
+      <c r="I1327" t="inlineStr"/>
+      <c r="J1327" t="inlineStr"/>
+      <c r="K1327" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1327" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>Live Academia</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://www.liveacademia.com.br</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr"/>
+      <c r="I1328" t="inlineStr"/>
+      <c r="J1328" t="inlineStr"/>
+      <c r="K1328" t="n">
+        <v>70</v>
+      </c>
+      <c r="L1328" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Centro-Oeste, +6 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1341"/>
+  <dimension ref="A1:L1347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65237,10 +65237,8 @@
         </is>
       </c>
       <c r="H1329" t="inlineStr"/>
-      <c r="I1329" t="inlineStr">
-        <is>
-          <t>5582993327839</t>
-        </is>
+      <c r="I1329" t="n">
+        <v>5582993327839</v>
       </c>
       <c r="J1329" t="inlineStr"/>
       <c r="K1329" t="n">
@@ -65385,10 +65383,8 @@
         </is>
       </c>
       <c r="H1332" t="inlineStr"/>
-      <c r="I1332" t="inlineStr">
-        <is>
-          <t>5582988510501</t>
-        </is>
+      <c r="I1332" t="n">
+        <v>5582988510501</v>
       </c>
       <c r="J1332" t="inlineStr"/>
       <c r="K1332" t="n">
@@ -65437,10 +65433,8 @@
         </is>
       </c>
       <c r="H1333" t="inlineStr"/>
-      <c r="I1333" t="inlineStr">
-        <is>
-          <t>551151989901</t>
-        </is>
+      <c r="I1333" t="n">
+        <v>551151989901</v>
       </c>
       <c r="J1333" t="inlineStr"/>
       <c r="K1333" t="n">
@@ -65489,10 +65483,8 @@
         </is>
       </c>
       <c r="H1334" t="inlineStr"/>
-      <c r="I1334" t="inlineStr">
-        <is>
-          <t>5571993786306</t>
-        </is>
+      <c r="I1334" t="n">
+        <v>5571993786306</v>
       </c>
       <c r="J1334" t="inlineStr"/>
       <c r="K1334" t="n">
@@ -65541,10 +65533,8 @@
         </is>
       </c>
       <c r="H1335" t="inlineStr"/>
-      <c r="I1335" t="inlineStr">
-        <is>
-          <t>5511945429541</t>
-        </is>
+      <c r="I1335" t="n">
+        <v>5511945429541</v>
       </c>
       <c r="J1335" t="inlineStr"/>
       <c r="K1335" t="n">
@@ -65641,10 +65631,8 @@
         </is>
       </c>
       <c r="H1337" t="inlineStr"/>
-      <c r="I1337" t="inlineStr">
-        <is>
-          <t>557131901041</t>
-        </is>
+      <c r="I1337" t="n">
+        <v>557131901041</v>
       </c>
       <c r="J1337" t="inlineStr"/>
       <c r="K1337" t="n">
@@ -65693,10 +65681,8 @@
         </is>
       </c>
       <c r="H1338" t="inlineStr"/>
-      <c r="I1338" t="inlineStr">
-        <is>
-          <t>5571996461571</t>
-        </is>
+      <c r="I1338" t="n">
+        <v>5571996461571</v>
       </c>
       <c r="J1338" t="inlineStr"/>
       <c r="K1338" t="n">
@@ -65745,10 +65731,8 @@
         </is>
       </c>
       <c r="H1339" t="inlineStr"/>
-      <c r="I1339" t="inlineStr">
-        <is>
-          <t>551140033273</t>
-        </is>
+      <c r="I1339" t="n">
+        <v>551140033273</v>
       </c>
       <c r="J1339" t="inlineStr"/>
       <c r="K1339" t="n">
@@ -65856,6 +65840,302 @@
         </is>
       </c>
     </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>Psicólogo em Brasília</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>https://buscadoutor.com.br</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr"/>
+      <c r="I1342" t="inlineStr"/>
+      <c r="J1342" t="inlineStr"/>
+      <c r="K1342" t="n">
+        <v>44</v>
+      </c>
+      <c r="L1342" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Venâncio Advocacia em Brasília</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>https://www.venancioadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr"/>
+      <c r="I1343" t="inlineStr"/>
+      <c r="J1343" t="inlineStr"/>
+      <c r="K1343" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1343" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>Clínica médica e check-up em Goiânia</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>https://drjosevictor.com</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr"/>
+      <c r="I1344" t="inlineStr"/>
+      <c r="J1344" t="inlineStr"/>
+      <c r="K1344" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1344" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>Musculação em Goiânia — Aula Experimental</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>https://athosacademia.com.br</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr"/>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>556232801214</t>
+        </is>
+      </c>
+      <c r="J1345" t="inlineStr"/>
+      <c r="K1345" t="n">
+        <v>70</v>
+      </c>
+      <c r="L1345" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>ABBA Fisioterapia em Goiânia</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>https://abbafisioterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr"/>
+      <c r="I1346" t="inlineStr"/>
+      <c r="J1346" t="inlineStr"/>
+      <c r="K1346" t="n">
+        <v>53</v>
+      </c>
+      <c r="L1346" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>Clínica de Fisioterapia Goiânia</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>https://antoniofisio.com</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr"/>
+      <c r="I1347" t="inlineStr">
+        <is>
+          <t>5562981040646</t>
+        </is>
+      </c>
+      <c r="J1347" t="inlineStr"/>
+      <c r="K1347" t="n">
+        <v>62</v>
+      </c>
+      <c r="L1347" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>